<commit_message>
Price list: cotton scarves (R35) on the Coin & Bright row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FrAdmZhbnvV2Pi8Ea2YxmY
</commit_message>
<xml_diff>
--- a/marketing/price-lists/Main_Price_List_with_online_prices_-_NOVEMBER_2026.xlsx
+++ b/marketing/price-lists/Main_Price_List_with_online_prices_-_NOVEMBER_2026.xlsx
@@ -6387,7 +6387,11 @@
           <t>R28-00</t>
         </is>
       </c>
-      <c r="G174" s="15" t="n"/>
+      <c r="G174" s="18" t="inlineStr">
+        <is>
+          <t>R35-00</t>
+        </is>
+      </c>
       <c r="H174" s="17" t="inlineStr">
         <is>
           <t>x1308</t>

</xml_diff>

<commit_message>
Price list: long WEB prices shrink to fit their cells
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FrAdmZhbnvV2Pi8Ea2YxmY
</commit_message>
<xml_diff>
--- a/marketing/price-lists/Main_Price_List_with_online_prices_-_NOVEMBER_2026.xlsx
+++ b/marketing/price-lists/Main_Price_List_with_online_prices_-_NOVEMBER_2026.xlsx
@@ -232,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -407,6 +407,22 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" shrinkToFit="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment shrinkToFit="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment shrinkToFit="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" shrinkToFit="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -783,6 +799,7 @@
     <col width="9.7109375" customWidth="1" style="2" min="2" max="2"/>
     <col width="7.42578125" customWidth="1" style="1" min="3" max="3"/>
     <col width="8.42578125" customWidth="1" style="1" min="4" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="8.28515625" customWidth="1" style="1" min="6" max="6"/>
     <col width="7.5703125" customWidth="1" style="1" min="7" max="7"/>
     <col width="6.28515625" customWidth="1" style="1" min="8" max="8"/>
@@ -2899,7 +2916,7 @@
           <t>R1030-00</t>
         </is>
       </c>
-      <c r="G65" s="18" t="inlineStr">
+      <c r="G65" s="52" t="inlineStr">
         <is>
           <t>R1135-00</t>
         </is>
@@ -2935,7 +2952,7 @@
           <t>R1000-00</t>
         </is>
       </c>
-      <c r="G66" s="18" t="inlineStr">
+      <c r="G66" s="52" t="inlineStr">
         <is>
           <t>R1100-00</t>
         </is>
@@ -3007,7 +3024,7 @@
           <t>R1030-00</t>
         </is>
       </c>
-      <c r="G68" s="18" t="inlineStr">
+      <c r="G68" s="52" t="inlineStr">
         <is>
           <t>R1135-00</t>
         </is>
@@ -3043,7 +3060,7 @@
           <t>R1000-00</t>
         </is>
       </c>
-      <c r="G69" s="18" t="inlineStr">
+      <c r="G69" s="52" t="inlineStr">
         <is>
           <t>R1100-00</t>
         </is>
@@ -3187,7 +3204,7 @@
           <t>R1030-00</t>
         </is>
       </c>
-      <c r="G73" s="18" t="inlineStr">
+      <c r="G73" s="52" t="inlineStr">
         <is>
           <t>R1135-00</t>
         </is>
@@ -4495,7 +4512,7 @@
           <t>R1050-00</t>
         </is>
       </c>
-      <c r="G108" s="49" t="inlineStr">
+      <c r="G108" s="53" t="inlineStr">
         <is>
           <t>R1150-00</t>
         </is>
@@ -5011,7 +5028,7 @@
           <t>R1010-00</t>
         </is>
       </c>
-      <c r="G124" s="18" t="inlineStr">
+      <c r="G124" s="52" t="inlineStr">
         <is>
           <t>R1115-00</t>
         </is>
@@ -5047,7 +5064,7 @@
           <t>R1135-00</t>
         </is>
       </c>
-      <c r="G125" s="18" t="inlineStr">
+      <c r="G125" s="52" t="inlineStr">
         <is>
           <t>R1250-00</t>
         </is>
@@ -7801,7 +7818,7 @@
           <t>R3-00</t>
         </is>
       </c>
-      <c r="G225" s="18" t="inlineStr">
+      <c r="G225" s="52" t="inlineStr">
         <is>
           <t>R30 for 10</t>
         </is>
@@ -10349,7 +10366,7 @@
           <t>R120/Dz</t>
         </is>
       </c>
-      <c r="G315" s="18" t="inlineStr">
+      <c r="G315" s="52" t="inlineStr">
         <is>
           <t>R15 each</t>
         </is>
@@ -10387,7 +10404,7 @@
           <t>R130/Dz</t>
         </is>
       </c>
-      <c r="G316" s="18" t="inlineStr">
+      <c r="G316" s="52" t="inlineStr">
         <is>
           <t>R15 each</t>
         </is>
@@ -10853,7 +10870,7 @@
           <t>R80/pkt</t>
         </is>
       </c>
-      <c r="G331" s="18" t="inlineStr">
+      <c r="G331" s="52" t="inlineStr">
         <is>
           <t>R95/pkt</t>
         </is>
@@ -11549,7 +11566,7 @@
           <t>R1150-00</t>
         </is>
       </c>
-      <c r="G357" s="18" t="inlineStr">
+      <c r="G357" s="52" t="inlineStr">
         <is>
           <t>R1150-00</t>
         </is>
@@ -11581,7 +11598,7 @@
           <t>R1320-00</t>
         </is>
       </c>
-      <c r="G358" s="18" t="inlineStr">
+      <c r="G358" s="52" t="inlineStr">
         <is>
           <t>R1320-00</t>
         </is>
@@ -12961,7 +12978,7 @@
           <t>R15 for 50</t>
         </is>
       </c>
-      <c r="G407" s="18" t="inlineStr">
+      <c r="G407" s="52" t="inlineStr">
         <is>
           <t>R20 for 50</t>
         </is>
@@ -13073,7 +13090,7 @@
           <t>R1100-00</t>
         </is>
       </c>
-      <c r="G411" s="18" t="inlineStr">
+      <c r="G411" s="52" t="inlineStr">
         <is>
           <t>R1100-00</t>
         </is>
@@ -13509,7 +13526,7 @@
           <t>R20-00</t>
         </is>
       </c>
-      <c r="G427" s="18" t="inlineStr">
+      <c r="G427" s="52" t="inlineStr">
         <is>
           <t>R10 hand / R15 leg</t>
         </is>

</xml_diff>

<commit_message>
Block Bath Towel R95 and thick matseka R25 (site waiting for upload, price list updated)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FrAdmZhbnvV2Pi8Ea2YxmY
</commit_message>
<xml_diff>
--- a/marketing/price-lists/Main_Price_List_with_online_prices_-_NOVEMBER_2026.xlsx
+++ b/marketing/price-lists/Main_Price_List_with_online_prices_-_NOVEMBER_2026.xlsx
@@ -5670,11 +5670,7 @@
           <t>R65-00</t>
         </is>
       </c>
-      <c r="G145" s="18" t="inlineStr">
-        <is>
-          <t>R75-00</t>
-        </is>
-      </c>
+      <c r="G145" s="18" t="n"/>
       <c r="H145" s="15" t="n"/>
     </row>
     <row r="146">
@@ -5700,7 +5696,11 @@
           <t>R85-00</t>
         </is>
       </c>
-      <c r="G146" s="15" t="n"/>
+      <c r="G146" s="18" t="inlineStr">
+        <is>
+          <t>R95-00</t>
+        </is>
+      </c>
       <c r="H146" s="15" t="n"/>
     </row>
     <row r="147">
@@ -13528,7 +13528,7 @@
       </c>
       <c r="G427" s="52" t="inlineStr">
         <is>
-          <t>R10 hand / R15 leg</t>
+          <t>R25-00</t>
         </is>
       </c>
       <c r="H427" s="15" t="n"/>

</xml_diff>

<commit_message>
Add Goleet Rings (set of 4, R250) to site build and price list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FrAdmZhbnvV2Pi8Ea2YxmY
</commit_message>
<xml_diff>
--- a/marketing/price-lists/Main_Price_List_with_online_prices_-_NOVEMBER_2026.xlsx
+++ b/marketing/price-lists/Main_Price_List_with_online_prices_-_NOVEMBER_2026.xlsx
@@ -14028,7 +14028,11 @@
           <t>R200-00</t>
         </is>
       </c>
-      <c r="G446" s="15" t="n"/>
+      <c r="G446" s="18" t="inlineStr">
+        <is>
+          <t>R250-00</t>
+        </is>
+      </c>
       <c r="H446" s="15" t="n"/>
     </row>
     <row r="447">

</xml_diff>